<commit_message>
Bilan promoteur: matrice habillée, téléchargeable, et simulateur recalé
Le classeur de la première série, encore signé Valora, passe aux couleurs
de CorpusImmo avec le logo et www.corpus.immo, sans tiret cadratin. Il est
téléchargeable depuis sa fiche, avec ses captures. Le simulateur gagne la
contre-épreuve complète et la grille de sensibilité, testées contre les
valeurs recalculées par Numbers. Les captures passent en v3 pour contourner
les caches, et les derniers tirets du DCF disparaissent.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/outils/matrices/dcf-valorisation.xlsx
+++ b/public/outils/matrices/dcf-valorisation.xlsx
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Rappel acquisition — Prix HD</t>
+          <t>Rappel acquisition : Prix HD</t>
         </is>
       </c>
       <c r="E10" s="16">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Rappel acquisition — Droits</t>
+          <t>Rappel acquisition : Droits</t>
         </is>
       </c>
       <c r="E11" s="16">
@@ -1151,7 +1151,7 @@
     <row r="12">
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Rappel acquisition — Fonds propres (= flux période 0)</t>
+          <t>Rappel acquisition : Fonds propres (= flux période 0)</t>
         </is>
       </c>
       <c r="E12" s="16">
@@ -1795,7 +1795,7 @@
       <c r="B30" s="6" t="n"/>
       <c r="D30" s="27" t="inlineStr">
         <is>
-          <t>Contrôle — % surface relouée (doit être ≤ 100%)</t>
+          <t>Contrôle : % surface relouée (doit être ≤ 100%)</t>
         </is>
       </c>
       <c r="E30" s="28">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D31" s="27" t="inlineStr">
         <is>
-          <t>Contrôle — % capex engagé (doit être = 100%)</t>
+          <t>Contrôle : % capex engagé (doit être = 100%)</t>
         </is>
       </c>
       <c r="E31" s="28">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="D32" s="27" t="inlineStr">
         <is>
-          <t>Contrôle — horizon de détention (doit être entre 1 et 7)</t>
+          <t>Contrôle : horizon de détention (doit être entre 1 et 7)</t>
         </is>
       </c>
       <c r="E32" s="8">
@@ -1996,7 +1996,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="32" t="inlineStr">
         <is>
-          <t>MATRICE DCF IMMOBILIER — MÉTHODE, CONVENTIONS ET LIMITES</t>
+          <t>MATRICE DCF IMMOBILIER : MÉTHODE, CONVENTIONS ET LIMITES</t>
         </is>
       </c>
       <c r="B1" s="32" t="n"/>
@@ -2131,7 +2131,7 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>— Il ne gère aucune échéance de bail : le loyer en place est supposé courir et s'indexer sur tout l'horizon, sans break ni expiration. Sur un actif tertiaire, c'est la simplification la plus lourde du modèle.</t>
+          <t>· Il ne gère aucune échéance de bail : le loyer en place est supposé courir et s'indexer sur tout l'horizon, sans break ni expiration. Sur un actif tertiaire, c'est la simplification la plus lourde du modèle.</t>
         </is>
       </c>
       <c r="B17" s="36" t="n"/>
@@ -2139,7 +2139,7 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="36" t="inlineStr">
         <is>
-          <t>— Il n'intègre ni fiscalité, ni impôt sur les sociétés, ni frais de structure ou d'asset management.</t>
+          <t>· Il n'intègre ni fiscalité, ni impôt sur les sociétés, ni frais de structure ou d'asset management.</t>
         </is>
       </c>
       <c r="B18" s="36" t="n"/>
@@ -2147,7 +2147,7 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>— Il ne traite ni les baux à paliers, ni les loyers variables, ni le détail des refacturations de charges.</t>
+          <t>· Il ne traite ni les baux à paliers, ni les loyers variables, ni le détail des refacturations de charges.</t>
         </is>
       </c>
       <c r="B19" s="36" t="n"/>
@@ -2155,7 +2155,7 @@
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="36" t="inlineStr">
         <is>
-          <t>— Il ne remplace pas une due diligence : état locatif réel, audit technique, urbanisme et environnement restent hors champ.</t>
+          <t>· Il ne remplace pas une due diligence : état locatif réel, audit technique, urbanisme et environnement restent hors champ.</t>
         </is>
       </c>
       <c r="B20" s="36" t="n"/>
@@ -2163,7 +2163,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>— L'horizon est limité à 7 périodes. Au-delà, aucune cession n'est simulée : la saisie est bloquée et un contrôle le signale.</t>
+          <t>· L'horizon est limité à 7 périodes. Au-delà, aucune cession n'est simulée : la saisie est bloquée et un contrôle le signale.</t>
         </is>
       </c>
       <c r="B21" s="36" t="n"/>

</xml_diff>